<commit_message>
added test senario T20
</commit_message>
<xml_diff>
--- a/SwatiRawat-testing-compose-function -Gmail.xlsx
+++ b/SwatiRawat-testing-compose-function -Gmail.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/96a1ec5e8d1ce7fb/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SWATI\pythonproj\Assignments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="101" documentId="8_{569B0172-5BBD-47ED-BCAD-0901C7EB5E5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD2CD841-2DAC-4D19-B8F2-90285E6B2A74}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7EBE354-5692-4B40-9C22-4E8A9AECDB94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{AAB91B10-3432-4B1B-8D38-4D1ACFA738CF}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="168">
   <si>
     <t>Gmail Compose – Functional Test Cases (Traditional)</t>
   </si>
@@ -1829,7 +1829,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75B74F74-FA7C-4932-8C89-45DDD70EC10A}">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -2075,6 +2075,11 @@
         <v>93</v>
       </c>
     </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" s="10" t="s">
+        <v>123</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:C1"/>

</xml_diff>